<commit_message>
chore: hapus "Cabang Senopati", pakai nama cabang aktif
- storeName default dikosongkan, mengikuti cabang aktif (Cimahi/Bandung)
- regenerate template database (.xlsx)
- update dokumen & log sesi
</commit_message>
<xml_diff>
--- a/templates-database/mycustomer-database-template.xlsx
+++ b/templates-database/mycustomer-database-template.xlsx
@@ -21071,11 +21071,7 @@
           <t>storeName</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Cabang Senopati</t>
-        </is>
-      </c>
+      <c r="B2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">

</xml_diff>